<commit_message>
Update <Mood disorder> and <Anxiety disorder> definitions
</commit_message>
<xml_diff>
--- a/terminology_resource.xlsx
+++ b/terminology_resource.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lauramenotti/Documents/Laura/RICERCA/PAPERS-PRESENTATIONS/2026/LREC/LREC26/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessa/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC49558C-2D6F-0E43-8CCA-82F76A099ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4357910-3AE5-2C45-A21C-9266875517DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" activeTab="3" xr2:uid="{AB8518AE-64E2-2842-81B9-E381C5C00868}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="25600" windowHeight="16000" xr2:uid="{AB8518AE-64E2-2842-81B9-E381C5C00868}"/>
   </bookViews>
   <sheets>
     <sheet name="Intensional Definitions" sheetId="1" r:id="rId1"/>
@@ -65,15 +65,6 @@
     <t>&lt;Mood disorder&gt;</t>
   </si>
   <si>
-    <t>psychiatric disorder constituting a category of disorders, characterized by anxious feeling or fear</t>
-  </si>
-  <si>
-    <t>psychiatric disorder constituting a category of disorders, characterized by disturbance in mood as their predominant feature</t>
-  </si>
-  <si>
-    <t>biota composed of the microorganisms (including bacteria, virus, archaea, and fungi) that exist in an organism</t>
-  </si>
-  <si>
     <t>microorganism that is unicellular, prokaryotic, and reproduces by cell division</t>
   </si>
   <si>
@@ -192,6 +183,15 @@
   </si>
   <si>
     <t>Embedded in the more general relation "is linked to"</t>
+  </si>
+  <si>
+    <t>mental disorder constituting a category of disorders, characterized by disturbance in mood as their predominant feature</t>
+  </si>
+  <si>
+    <t>mental disorder constituting a category of disorders, characterized by anxious feeling or fear</t>
+  </si>
+  <si>
+    <t>biota composed of microorganisms, including bacteria, virus, archaea and fungi, that exist in an organism</t>
   </si>
 </sst>
 </file>
@@ -270,7 +270,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -287,6 +287,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -631,10 +634,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -642,15 +645,15 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
+      <c r="B3" s="12" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="35" customHeight="1" x14ac:dyDescent="0.2">
@@ -658,7 +661,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -666,7 +669,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -674,7 +677,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -682,7 +685,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -690,7 +693,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>8</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.2">
@@ -698,7 +701,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -738,90 +741,90 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -857,13 +860,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="57" customHeight="1" x14ac:dyDescent="0.2">
@@ -871,10 +874,10 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -882,10 +885,10 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -893,10 +896,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -904,10 +907,10 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -915,10 +918,10 @@
         <v>6</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -926,10 +929,10 @@
         <v>7</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -955,112 +958,112 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>